<commit_message>
promovix-figma: colunas em promoção no visual da proposta 1
Escolhida pelo Otávio entre 6 propostas visuais: faixa amarelo-clara
contínua atrás das colunas em promoção, preço em oferta em negrito e
adesivo preto/amarelo sobre a borda da tabela (texto em adesivo_promo
no Config, padrão "REFLECTA −50%"). A altura da faixa é refeita no fim,
depois do respiro e do aperto da página.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/plugins/vixlens-catalogo/skills/promovix-figma/modelo/Promovix_modelo.xlsx
+++ b/plugins/vixlens-catalogo/skills/promovix-figma/modelo/Promovix_modelo.xlsx
@@ -458,9 +458,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -542,7 +540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -869,6 +867,23 @@
       <c r="C19" s="4" t="inlineStr">
         <is>
           <t>Capa.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>adesivo_promo</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>REFLECTA −50%</t>
+        </is>
+      </c>
+      <c r="C20" s="4" t="inlineStr">
+        <is>
+          <t>Adesivo preto sobre as colunas em promoção (colunas_promo). Vazio = sem adesivo.</t>
         </is>
       </c>
     </row>
@@ -1239,7 +1254,6 @@
           <t>Sem A.R.;A.R. Eco;Reflecta Express</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>N</t>
@@ -1255,7 +1269,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr"/>
       <c r="K2" t="n">
         <v>70</v>
       </c>
@@ -1291,7 +1304,6 @@
           <t>Sem A.R.;Reflecta Express;Reflecta Guard</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr">
         <is>
           <t>N</t>
@@ -1307,7 +1319,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr"/>
       <c r="K3" t="n">
         <v>70</v>
       </c>
@@ -1343,7 +1354,6 @@
           <t>Sem A.R.;Reflecta Express;Reflecta Guard</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr">
         <is>
           <t>N</t>
@@ -1359,7 +1369,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr"/>
       <c r="K4" t="n">
         <v>70</v>
       </c>
@@ -1385,13 +1394,11 @@
           <t>#DADFE2</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>Par</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
         <is>
           <t>N</t>
@@ -1467,7 +1474,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr"/>
       <c r="K6" t="n">
         <v>70</v>
       </c>
@@ -1523,7 +1529,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
       <c r="K7" t="n">
         <v>70</v>
       </c>
@@ -1579,7 +1584,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr"/>
       <c r="K8" t="n">
         <v>70</v>
       </c>
@@ -1635,7 +1639,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J9" t="inlineStr"/>
       <c r="K9" t="n">
         <v>70</v>
       </c>
@@ -1691,7 +1694,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J10" t="inlineStr"/>
       <c r="K10" t="n">
         <v>70</v>
       </c>
@@ -1747,7 +1749,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr"/>
       <c r="K11" t="n">
         <v>70</v>
       </c>
@@ -1803,7 +1804,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J12" t="inlineStr"/>
       <c r="K12" t="n">
         <v>70</v>
       </c>
@@ -1859,7 +1859,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J13" t="inlineStr"/>
       <c r="K13" t="n">
         <v>70</v>
       </c>
@@ -1885,13 +1884,11 @@
           <t>#D0DDE4</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>Par</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
           <t>N</t>
@@ -1907,7 +1904,6 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J14" t="inlineStr"/>
       <c r="K14" t="n">
         <v>92</v>
       </c>
@@ -1933,13 +1929,11 @@
           <t>#D0DDE4</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>Par</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
           <t>N</t>
@@ -1955,7 +1949,6 @@
           <t>S</t>
         </is>
       </c>
-      <c r="J15" t="inlineStr"/>
       <c r="K15" t="n">
         <v>92</v>
       </c>
@@ -1981,13 +1974,11 @@
           <t>#006BB2</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>Par</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr">
         <is>
           <t>N</t>
@@ -2003,7 +1994,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J16" t="inlineStr"/>
       <c r="K16" t="n">
         <v>95</v>
       </c>
@@ -2029,13 +2019,11 @@
           <t>#006BB2</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>Par</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr">
         <is>
           <t>N</t>
@@ -2051,7 +2039,6 @@
           <t>N</t>
         </is>
       </c>
-      <c r="J17" t="inlineStr"/>
       <c r="K17" t="n">
         <v>95</v>
       </c>
@@ -2494,7 +2481,6 @@
           <t>VIX TOTAL</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" t="inlineStr">
         <is>
           <t>1.49</t>
@@ -2731,7 +2717,6 @@
           <t>VIX TOTAL</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
       <c r="C14" t="inlineStr">
         <is>
           <t>1.59</t>
@@ -2960,7 +2945,6 @@
           <t>FREEVIX VISÃO SIMPLES</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr"/>
       <c r="C20" t="inlineStr">
         <is>
           <t>1.49</t>
@@ -3179,7 +3163,6 @@
           <t>FREEVIX VISÃO SIMPLES</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr"/>
       <c r="C26" t="inlineStr">
         <is>
           <t>1.59</t>
@@ -3605,7 +3588,6 @@
           <t>ESPACE PLUS DIGITAL</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr"/>
       <c r="C38" t="inlineStr">
         <is>
           <t>1.50</t>
@@ -3678,7 +3660,6 @@
           <t>ESPACE PLUS DIGITAL</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
       <c r="C40" t="inlineStr">
         <is>
           <t>1.59</t>
@@ -3782,7 +3763,6 @@
           <t>KODAK PRECISE NEXT</t>
         </is>
       </c>
-      <c r="B43" t="inlineStr"/>
       <c r="C43" t="inlineStr">
         <is>
           <t>1.50</t>
@@ -3855,7 +3835,6 @@
           <t>KODAK PRECISE NEXT</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
           <t>1.59</t>
@@ -3931,7 +3910,6 @@
           <t>KODAK PRECISE NEXT</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
           <t>1.67</t>
@@ -4038,7 +4016,6 @@
           <t>KODAK NETWORK UHD</t>
         </is>
       </c>
-      <c r="B50" t="inlineStr"/>
       <c r="C50" t="inlineStr">
         <is>
           <t>1.50</t>
@@ -4152,7 +4129,6 @@
           <t>KODAK NETWORK UHD</t>
         </is>
       </c>
-      <c r="B53" t="inlineStr"/>
       <c r="C53" t="inlineStr">
         <is>
           <t>1.59</t>
@@ -4269,7 +4245,6 @@
           <t>KODAK NETWORK UHD</t>
         </is>
       </c>
-      <c r="B56" t="inlineStr"/>
       <c r="C56" t="inlineStr">
         <is>
           <t>1.67</t>
@@ -4487,7 +4462,6 @@
           <t>KODAK UNIQUE UHD</t>
         </is>
       </c>
-      <c r="B62" t="inlineStr"/>
       <c r="C62" t="inlineStr">
         <is>
           <t>1.50</t>
@@ -4601,7 +4575,6 @@
           <t>KODAK UNIQUE UHD</t>
         </is>
       </c>
-      <c r="B65" t="inlineStr"/>
       <c r="C65" t="inlineStr">
         <is>
           <t>1.59</t>
@@ -4718,7 +4691,6 @@
           <t>KODAK UNIQUE UHD</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr"/>
       <c r="C68" t="inlineStr">
         <is>
           <t>1.67</t>
@@ -4825,7 +4797,6 @@
           <t>KODAK UNIQUE INFINITE</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr"/>
       <c r="C71" t="inlineStr">
         <is>
           <t>1.50</t>
@@ -4939,7 +4910,6 @@
           <t>KODAK UNIQUE INFINITE</t>
         </is>
       </c>
-      <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
           <t>1.59</t>
@@ -5056,7 +5026,6 @@
           <t>KODAK UNIQUE INFINITE</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr"/>
       <c r="C77" t="inlineStr">
         <is>
           <t>1.67</t>
@@ -5163,7 +5132,6 @@
           <t>KODAK SINGLE</t>
         </is>
       </c>
-      <c r="B80" t="inlineStr"/>
       <c r="C80" t="inlineStr">
         <is>
           <t>1.50</t>
@@ -5277,7 +5245,6 @@
           <t>KODAK SINGLE</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr"/>
       <c r="C83" t="inlineStr">
         <is>
           <t>1.59</t>
@@ -5394,7 +5361,6 @@
           <t>KODAK SINGLE</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr"/>
       <c r="C86" t="inlineStr">
         <is>
           <t>1.67</t>
@@ -5501,7 +5467,6 @@
           <t>ESSILOR SURFAÇADAS</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr"/>
       <c r="C89" t="inlineStr">
         <is>
           <t>1.50</t>
@@ -5605,7 +5570,6 @@
           <t>ESSILOR SURFAÇADAS</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr"/>
       <c r="C92" t="inlineStr">
         <is>
           <t>1.59</t>

</xml_diff>